<commit_message>
Add project files for AI course analysis, including data processing scripts, quality assessment, and documentation. Update .gitignore to exclude new directories and files. Introduce new datasets for simulation and analysis.
</commit_message>
<xml_diff>
--- a/Agenda_Distribuição_Topicos.xlsx
+++ b/Agenda_Distribuição_Topicos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bayergroup-my.sharepoint.com/personal/eder_silva_bayer_com/Documents/Share_Files/Curso_AI_UFV_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{DC84EE2C-98E1-49D1-A322-7AFE8E3A7A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBDADE37-10A2-4BC8-BE4D-623408566C2C}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{DC84EE2C-98E1-49D1-A322-7AFE8E3A7A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FACA037-2E91-4006-AFF4-B18B6CF2A345}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="6375" windowWidth="29040" windowHeight="15720" xr2:uid="{4614778F-B9C0-456D-A2D7-C01AD282FF12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4614778F-B9C0-456D-A2D7-C01AD282FF12}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -309,12 +309,19 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -327,13 +334,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -672,12 +672,12 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="66.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.85546875" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" customWidth="1"/>
     <col min="5" max="5" width="20.140625" customWidth="1"/>
-    <col min="6" max="6" width="44.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -690,27 +690,27 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+      <c r="A2" s="9">
         <v>46092</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="13"/>
+      <c r="D2" s="7"/>
       <c r="E2" t="s">
         <v>8</v>
       </c>
@@ -719,12 +719,12 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="10"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="13"/>
+      <c r="D3" s="7"/>
       <c r="E3" t="s">
         <v>9</v>
       </c>
@@ -733,12 +733,12 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="13"/>
+      <c r="D4" s="7"/>
       <c r="E4" t="s">
         <v>10</v>
       </c>
@@ -747,12 +747,12 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="11"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="13"/>
+      <c r="D5" s="7"/>
       <c r="E5" t="s">
         <v>11</v>
       </c>
@@ -770,7 +770,7 @@
       <c r="C6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="13"/>
+      <c r="D6" s="7"/>
       <c r="E6" t="s">
         <v>11</v>
       </c>
@@ -779,16 +779,16 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>46123</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="7"/>
       <c r="E7" t="s">
         <v>16</v>
       </c>
@@ -796,13 +796,13 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="11"/>
+    <row r="8" spans="1:6" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="13"/>
+      <c r="D8" s="7"/>
       <c r="E8" t="s">
         <v>9</v>
       </c>
@@ -811,16 +811,16 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>46123</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="13"/>
+      <c r="D9" s="7"/>
       <c r="E9" t="s">
         <v>18</v>
       </c>
@@ -829,12 +829,12 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="11"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="14"/>
       <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="13"/>
+      <c r="D10" s="7"/>
       <c r="E10" t="s">
         <v>23</v>
       </c>
@@ -852,7 +852,7 @@
       <c r="C11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="13"/>
+      <c r="D11" s="7"/>
       <c r="E11" t="s">
         <v>8</v>
       </c>
@@ -870,7 +870,7 @@
       <c r="C12" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="13"/>
+      <c r="D12" s="7"/>
       <c r="E12" t="s">
         <v>21</v>
       </c>
@@ -884,7 +884,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="8" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>